<commit_message>
hakediş genel bilgile güncellendi
</commit_message>
<xml_diff>
--- a/views/hakedisler/Hakedis.xlsx
+++ b/views/hakedisler/Hakedis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\ersan_elk\views\hakedisler\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5F843B1-D99C-47B2-B1FE-BDAA284BA3B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81A43A47-0F7D-4700-B27B-2D81558FBE84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="918" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="918" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bilgiler" sheetId="1" r:id="rId1"/>
@@ -19063,15 +19063,11 @@
       <c r="E10" s="502"/>
       <c r="F10" s="502"/>
       <c r="G10" s="502"/>
-      <c r="H10" s="608">
-        <v>2025</v>
-      </c>
+      <c r="H10" s="608"/>
       <c r="I10" s="608"/>
       <c r="J10" s="608"/>
       <c r="K10" s="608"/>
-      <c r="L10" s="502">
-        <v>2026</v>
-      </c>
+      <c r="L10" s="502"/>
       <c r="M10" s="502"/>
       <c r="N10" s="502"/>
       <c r="O10" s="502"/>
@@ -19098,10 +19094,7 @@
       <c r="E11" s="602"/>
       <c r="F11" s="602"/>
       <c r="G11" s="602"/>
-      <c r="H11" s="531">
-        <f>'İş Takip-Ön Yüz'!G14</f>
-        <v>0</v>
-      </c>
+      <c r="H11" s="531"/>
       <c r="I11" s="498"/>
       <c r="J11" s="498"/>
       <c r="K11" s="498"/>
@@ -19132,10 +19125,7 @@
       <c r="E12" s="602"/>
       <c r="F12" s="602"/>
       <c r="G12" s="602"/>
-      <c r="H12" s="531">
-        <f>'Arka Kapak'!D4</f>
-        <v>0</v>
-      </c>
+      <c r="H12" s="531"/>
       <c r="I12" s="531"/>
       <c r="J12" s="531"/>
       <c r="K12" s="531"/>

</xml_diff>

<commit_message>
hakedişş ve araç yakıt güncellemeleri
</commit_message>
<xml_diff>
--- a/views/hakedisler/Hakedis.xlsx
+++ b/views/hakedisler/Hakedis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\ersan_elk\views\hakedisler\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81A43A47-0F7D-4700-B27B-2D81558FBE84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6774FE25-0157-4B08-9FAF-99684B5F53AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="918" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="918" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bilgiler" sheetId="1" r:id="rId1"/>

</xml_diff>